<commit_message>
feat(F-NAR-019): polish TREE-DIF-068 et TREE-AUT-009 xlsx
Alignement xlsx sur merged vocal après re-apply.
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-AUT-009.xlsx
+++ b/stories/arbres/TREE-AUT-009.xlsx
@@ -2739,17 +2739,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la cuisine, un peu lourd. Le matin, les cubes dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont une place, près du pain. Ils ont une place, le matin ! Le quai du tapis peut attendre dehors. Une miette de matin colle à la dent dorée.</t>
+          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la cuisine, un peu lourd. Le matin, les cubes dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont une place, près du pain. Ils ont une place, le matin ! Le quai du tapis peut attendre dehors. Une miette de matin colle à la dent dorée.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la cuisine, un peu lourd. Le matin, les cubes dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont une place, près du pain. Ils ont une place, le matin ! Le quai du tapis peut attendre dehors. Une miette de matin colle à la dent dorée.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la cuisine, un peu lourd. Le matin, les cubes dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont une place, près du pain. Ils ont une place, le matin ! Le quai du tapis peut attendre dehors. Une miette de matin colle à la dent dorée.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la cuisine, un peu lourd. Le matin, les cubes dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont une place, près du pain. Ils ont une place, le matin ! Le quai du tapis peut attendre dehors. Une miette de matin colle à la dent dorée. [pause]</t>
+          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la cuisine, un peu lourd. Le matin, les cubes dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont une place, près du pain. Ils ont une place, le matin ! Le quai du tapis peut attendre dehors. Une miette de matin colle à la dent dorée. [pause]</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino glisse un cube, puis l'autre, à plat.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|Tes cubes ont une place, près du pain.
 enfant-m|Ils ont une place, le matin !
 maman|Le quai du tapis peut attendre dehors.
@@ -3108,17 +3108,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la cuisine, un peu lourd. Après la sieste, les cubes dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont attendu la sieste, au chaud. Ils ont une place, après la sieste ! Le quai du tapis peut attendre dehors. Un cube tiède attend, sous la dent dorée.</t>
+          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la cuisine, un peu lourd. Après la sieste, les cubes dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont attendu la sieste, au chaud. Ils ont une place, après la sieste ! Le quai du tapis peut attendre dehors. Un cube tiède attend, sous la dent dorée.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la cuisine, un peu lourd. Après la sieste, les cubes dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont attendu la sieste, au chaud. Ils ont une place, après la sieste ! Le quai du tapis peut attendre dehors. Un cube tiède attend, sous la dent dorée.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la cuisine, un peu lourd. Après la sieste, les cubes dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont attendu la sieste, au chaud. Ils ont une place, après la sieste ! Le quai du tapis peut attendre dehors. Un cube tiède attend, sous la dent dorée.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la cuisine, un peu lourd. Après la sieste, les cubes dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont attendu la sieste, au chaud. Ils ont une place, après la sieste ! Le quai du tapis peut attendre dehors. Un cube tiède attend, sous la dent dorée. [pause]</t>
+          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la cuisine, un peu lourd. Après la sieste, les cubes dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont attendu la sieste, au chaud. Ils ont une place, après la sieste ! Le quai du tapis peut attendre dehors. Un cube tiède attend, sous la dent dorée. [pause]</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -3259,7 +3259,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino glisse un cube, puis l'autre, à plat.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|Tes cubes ont attendu la sieste, au chaud.
 enfant-m|Ils ont une place, après la sieste !
 maman|Le quai du tapis peut attendre dehors.
@@ -3481,17 +3481,17 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la cuisine, un peu lourd. Le soir, les cubes dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont une place, sous la lampe. Ils ont une place, le soir ! Le quai du tapis peut attendre dehors. La lampe allume un cube, derrière la dent.</t>
+          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la cuisine, un peu lourd. Le soir, les cubes dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont une place, sous la lampe. Ils ont une place, le soir ! Le quai du tapis peut attendre dehors. La lampe allume un cube, derrière la dent.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la cuisine, un peu lourd. Le soir, les cubes dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont une place, sous la lampe. Ils ont une place, le soir ! Le quai du tapis peut attendre dehors. La lampe allume un cube, derrière la dent.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la cuisine, un peu lourd. Le soir, les cubes dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont une place, sous la lampe. Ils ont une place, le soir ! Le quai du tapis peut attendre dehors. La lampe allume un cube, derrière la dent.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la cuisine, un peu lourd. Le soir, les cubes dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont une place, sous la lampe. Ils ont une place, le soir ! Le quai du tapis peut attendre dehors. La lampe allume un cube, derrière la dent. [pause]</t>
+          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la cuisine, un peu lourd. Le soir, les cubes dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont une place, sous la lampe. Ils ont une place, le soir ! Le quai du tapis peut attendre dehors. La lampe allume un cube, derrière la dent. [pause]</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -3632,7 +3632,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino glisse un cube, puis l'autre, à plat.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|Tes cubes ont une place, sous la lampe.
 enfant-m|Ils ont une place, le soir !
 maman|Le quai du tapis peut attendre dehors.
@@ -4240,17 +4240,17 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la cuisine, un peu lourd. Le matin, le livre dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a une place, près du four. Il a une place, le matin ! Le quai du tapis peut attendre dehors. Une page de matin sent le pain, au fond.</t>
+          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la cuisine, un peu lourd. Le matin, le livre dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a une place, près du four. Il a une place, le matin ! Le quai du tapis peut attendre dehors. Une page de matin sent le pain, au fond.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la cuisine, un peu lourd. Le matin, le livre dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a une place, près du four. Il a une place, le matin ! Le quai du tapis peut attendre dehors. Une page de matin sent le pain, au fond.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la cuisine, un peu lourd. Le matin, le livre dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a une place, près du four. Il a une place, le matin ! Le quai du tapis peut attendre dehors. Une page de matin sent le pain, au fond.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la cuisine, un peu lourd. Le matin, le livre dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a une place, près du four. Il a une place, le matin ! Le quai du tapis peut attendre dehors. Une page de matin sent le pain, au fond. [pause]</t>
+          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la cuisine, un peu lourd. Le matin, le livre dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a une place, près du four. Il a une place, le matin ! Le quai du tapis peut attendre dehors. Une page de matin sent le pain, au fond. [pause]</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -4391,7 +4391,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino couche le livre, pages vers le fond.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|Le livre a une place, près du four.
 enfant-m|Il a une place, le matin !
 maman|Le quai du tapis peut attendre dehors.
@@ -4609,17 +4609,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la cuisine, un peu lourd. Après la sieste, le livre dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a attendu le rideau, à plat. Il a une place, après la sieste ! Le quai du tapis peut attendre dehors. Le livre fait un toit, sous le rideau.</t>
+          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la cuisine, un peu lourd. Après la sieste, le livre dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a attendu le rideau, à plat. Il a une place, après la sieste ! Le quai du tapis peut attendre dehors. Le livre fait un toit, sous le rideau.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la cuisine, un peu lourd. Après la sieste, le livre dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a attendu le rideau, à plat. Il a une place, après la sieste ! Le quai du tapis peut attendre dehors. Le livre fait un toit, sous le rideau.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la cuisine, un peu lourd. Après la sieste, le livre dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a attendu le rideau, à plat. Il a une place, après la sieste ! Le quai du tapis peut attendre dehors. Le livre fait un toit, sous le rideau.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la cuisine, un peu lourd. Après la sieste, le livre dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a attendu le rideau, à plat. Il a une place, après la sieste ! Le quai du tapis peut attendre dehors. Le livre fait un toit, sous le rideau. [pause]</t>
+          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la cuisine, un peu lourd. Après la sieste, le livre dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a attendu le rideau, à plat. Il a une place, après la sieste ! Le quai du tapis peut attendre dehors. Le livre fait un toit, sous le rideau. [pause]</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -4760,7 +4760,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino couche le livre, pages vers le fond.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|Le livre a attendu le rideau, à plat.
 enfant-m|Il a une place, après la sieste !
 maman|Le quai du tapis peut attendre dehors.
@@ -4982,17 +4982,17 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la cuisine, un peu lourd. Le soir, le livre dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a une place, sous la lampe. Il a une place, le soir ! Le quai du tapis peut attendre dehors. La lampe glisse sur la couverture du livre.</t>
+          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la cuisine, un peu lourd. Le soir, le livre dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a une place, sous la lampe. Il a une place, le soir ! Le quai du tapis peut attendre dehors. La lampe glisse sur la couverture du livre.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la cuisine, un peu lourd. Le soir, le livre dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a une place, sous la lampe. Il a une place, le soir ! Le quai du tapis peut attendre dehors. La lampe glisse sur la couverture du livre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la cuisine, un peu lourd. Le soir, le livre dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a une place, sous la lampe. Il a une place, le soir ! Le quai du tapis peut attendre dehors. La lampe glisse sur la couverture du livre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la cuisine, un peu lourd. Le soir, le livre dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a une place, sous la lampe. Il a une place, le soir ! Le quai du tapis peut attendre dehors. La lampe glisse sur la couverture du livre. [pause]</t>
+          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la cuisine, un peu lourd. Le soir, le livre dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a une place, sous la lampe. Il a une place, le soir ! Le quai du tapis peut attendre dehors. La lampe glisse sur la couverture du livre. [pause]</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -5133,7 +5133,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino couche le livre, pages vers le fond.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|Le livre a une place, sous la lampe.
 enfant-m|Il a une place, le soir !
 maman|Le quai du tapis peut attendre dehors.
@@ -5741,17 +5741,17 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la cuisine, un peu lourd. Le matin, la tasse dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a une place, près du pain. Elle a une place, le matin ! Le quai du tapis peut attendre dehors. La tasse du matin sonne, toute petite.</t>
+          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la cuisine, un peu lourd. Le matin, la tasse dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a une place, près du pain. Elle a une place, le matin ! Le quai du tapis peut attendre dehors. La tasse du matin sonne, toute petite.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la cuisine, un peu lourd. Le matin, la tasse dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a une place, près du pain. Elle a une place, le matin ! Le quai du tapis peut attendre dehors. La tasse du matin sonne, toute petite.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la cuisine, un peu lourd. Le matin, la tasse dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a une place, près du pain. Elle a une place, le matin ! Le quai du tapis peut attendre dehors. La tasse du matin sonne, toute petite.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la cuisine, un peu lourd. Le matin, la tasse dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a une place, près du pain. Elle a une place, le matin ! Le quai du tapis peut attendre dehors. La tasse du matin sonne, toute petite. [pause]</t>
+          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la cuisine, un peu lourd. Le matin, la tasse dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a une place, près du pain. Elle a une place, le matin ! Le quai du tapis peut attendre dehors. La tasse du matin sonne, toute petite. [pause]</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -5892,7 +5892,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino niche la tasse, contre le doudou.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|La tasse a une place, près du pain.
 enfant-m|Elle a une place, le matin !
 maman|Le quai du tapis peut attendre dehors.
@@ -6110,17 +6110,17 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la cuisine, un peu lourd. Après la sieste, la tasse dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a attendu, sans rouler. Elle a une place, après la sieste ! Le quai du tapis peut attendre dehors. La tasse de sieste ne roule plus.</t>
+          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la cuisine, un peu lourd. Après la sieste, la tasse dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a attendu, sans rouler. Elle a une place, après la sieste ! Le quai du tapis peut attendre dehors. La tasse de sieste ne roule plus.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la cuisine, un peu lourd. Après la sieste, la tasse dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a attendu, sans rouler. Elle a une place, après la sieste ! Le quai du tapis peut attendre dehors. La tasse de sieste ne roule plus.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la cuisine, un peu lourd. Après la sieste, la tasse dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a attendu, sans rouler. Elle a une place, après la sieste ! Le quai du tapis peut attendre dehors. La tasse de sieste ne roule plus.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la cuisine, un peu lourd. Après la sieste, la tasse dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a attendu, sans rouler. Elle a une place, après la sieste ! Le quai du tapis peut attendre dehors. La tasse de sieste ne roule plus. [pause]</t>
+          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la cuisine, un peu lourd. Après la sieste, la tasse dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a attendu, sans rouler. Elle a une place, après la sieste ! Le quai du tapis peut attendre dehors. La tasse de sieste ne roule plus. [pause]</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -6261,7 +6261,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino niche la tasse, contre le doudou.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|La tasse a attendu, sans rouler.
 enfant-m|Elle a une place, après la sieste !
 maman|Le quai du tapis peut attendre dehors.
@@ -6483,17 +6483,17 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la cuisine, un peu lourd. Le soir, la tasse dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a une place, sous la lampe. Elle a une place, le soir ! Le quai du tapis peut attendre dehors. La tasse du soir cache un reflet de lampe.</t>
+          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la cuisine, un peu lourd. Le soir, la tasse dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a une place, sous la lampe. Elle a une place, le soir ! Le quai du tapis peut attendre dehors. La tasse du soir cache un reflet de lampe.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la cuisine, un peu lourd. Le soir, la tasse dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a une place, sous la lampe. Elle a une place, le soir ! Le quai du tapis peut attendre dehors. La tasse du soir cache un reflet de lampe.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la cuisine, un peu lourd. Le soir, la tasse dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a une place, sous la lampe. Elle a une place, le soir ! Le quai du tapis peut attendre dehors. La tasse du soir cache un reflet de lampe.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la cuisine, un peu lourd. Le soir, la tasse dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a une place, sous la lampe. Elle a une place, le soir ! Le quai du tapis peut attendre dehors. La tasse du soir cache un reflet de lampe. [pause]</t>
+          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la cuisine, un peu lourd. Le soir, la tasse dans le sac ! Le pain a failli rester sur la chaise. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a une place, sous la lampe. Elle a une place, le soir ! Le quai du tapis peut attendre dehors. La tasse du soir cache un reflet de lampe. [pause]</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -6634,7 +6634,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino niche la tasse, contre le doudou.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|La tasse a une place, sous la lampe.
 enfant-m|Elle a une place, le soir !
 maman|Le quai du tapis peut attendre dehors.
@@ -8000,17 +8000,17 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est près du jardin, un peu lourd. Le matin, les cubes dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont une place, malgré l'herbe. Ils ont une place, le matin ! Le quai du tapis peut attendre dehors. Un cube d'herbe sèche, contre la dent dorée.</t>
+          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est près du jardin, un peu lourd. Le matin, les cubes dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont une place, malgré l'herbe. Ils ont une place, le matin ! Le quai du tapis peut attendre dehors. Un cube d'herbe sèche, contre la dent dorée.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au matin, la lumière est fraîche, près de la porte. Le sac bleu est près du jardin, un peu lourd. Le matin, les cubes dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont une place, malgré l'herbe. Ils ont une place, le matin ! Le quai du tapis peut attendre dehors. Un cube d'herbe sèche, contre la dent dorée.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au matin, la lumière est fraîche, près de la porte. Le sac bleu est près du jardin, un peu lourd. Le matin, les cubes dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont une place, malgré l'herbe. Ils ont une place, le matin ! Le quai du tapis peut attendre dehors. Un cube d'herbe sèche, contre la dent dorée.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est près du jardin, un peu lourd. Le matin, les cubes dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont une place, malgré l'herbe. Ils ont une place, le matin ! Le quai du tapis peut attendre dehors. Un cube d'herbe sèche, contre la dent dorée. [pause]</t>
+          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est près du jardin, un peu lourd. Le matin, les cubes dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont une place, malgré l'herbe. Ils ont une place, le matin ! Le quai du tapis peut attendre dehors. Un cube d'herbe sèche, contre la dent dorée. [pause]</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
@@ -8151,7 +8151,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino glisse un cube, puis l'autre, à plat.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|Tes cubes ont une place, malgré l'herbe.
 enfant-m|Ils ont une place, le matin !
 maman|Le quai du tapis peut attendre dehors.
@@ -8369,17 +8369,17 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est près du jardin, un peu lourd. Après la sieste, les cubes dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont séché, pendant la sieste. Ils ont une place, après la sieste ! Le quai du tapis peut attendre dehors. Un cube tiède sent la dalle, au fond.</t>
+          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est près du jardin, un peu lourd. Après la sieste, les cubes dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont séché, pendant la sieste. Ils ont une place, après la sieste ! Le quai du tapis peut attendre dehors. Un cube tiède sent la dalle, au fond.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Après la sieste, le rideau fait un carré chaud. Le sac bleu est près du jardin, un peu lourd. Après la sieste, les cubes dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont séché, pendant la sieste. Ils ont une place, après la sieste ! Le quai du tapis peut attendre dehors. Un cube tiède sent la dalle, au fond.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Après la sieste, le rideau fait un carré chaud. Le sac bleu est près du jardin, un peu lourd. Après la sieste, les cubes dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont séché, pendant la sieste. Ils ont une place, après la sieste ! Le quai du tapis peut attendre dehors. Un cube tiède sent la dalle, au fond.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est près du jardin, un peu lourd. Après la sieste, les cubes dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont séché, pendant la sieste. Ils ont une place, après la sieste ! Le quai du tapis peut attendre dehors. Un cube tiède sent la dalle, au fond. [pause]</t>
+          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est près du jardin, un peu lourd. Après la sieste, les cubes dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont séché, pendant la sieste. Ils ont une place, après la sieste ! Le quai du tapis peut attendre dehors. Un cube tiède sent la dalle, au fond. [pause]</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
@@ -8520,7 +8520,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino glisse un cube, puis l'autre, à plat.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|Tes cubes ont séché, pendant la sieste.
 enfant-m|Ils ont une place, après la sieste !
 maman|Le quai du tapis peut attendre dehors.
@@ -8742,17 +8742,17 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est près du jardin, un peu lourd. Le soir, les cubes dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont une place, malgré le soir. Ils ont une place, le soir ! Le quai du tapis peut attendre dehors. Un cube du soir garde une poussière d'herbe.</t>
+          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est près du jardin, un peu lourd. Le soir, les cubes dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont une place, malgré le soir. Ils ont une place, le soir ! Le quai du tapis peut attendre dehors. Un cube du soir garde une poussière d'herbe.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, la lampe allume le tapis, tout près. Le sac bleu est près du jardin, un peu lourd. Le soir, les cubes dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont une place, malgré le soir. Ils ont une place, le soir ! Le quai du tapis peut attendre dehors. Un cube du soir garde une poussière d'herbe.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, la lampe allume le tapis, tout près. Le sac bleu est près du jardin, un peu lourd. Le soir, les cubes dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont une place, malgré le soir. Ils ont une place, le soir ! Le quai du tapis peut attendre dehors. Un cube du soir garde une poussière d'herbe.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est près du jardin, un peu lourd. Le soir, les cubes dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont une place, malgré le soir. Ils ont une place, le soir ! Le quai du tapis peut attendre dehors. Un cube du soir garde une poussière d'herbe. [pause]</t>
+          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est près du jardin, un peu lourd. Le soir, les cubes dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont une place, malgré le soir. Ils ont une place, le soir ! Le quai du tapis peut attendre dehors. Un cube du soir garde une poussière d'herbe. [pause]</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -8893,7 +8893,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino glisse un cube, puis l'autre, à plat.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|Tes cubes ont une place, malgré le soir.
 enfant-m|Ils ont une place, le soir !
 maman|Le quai du tapis peut attendre dehors.
@@ -9501,17 +9501,17 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est près du jardin, un peu lourd. Le matin, le livre dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a une place, malgré le vent. Il a une place, le matin ! Le quai du tapis peut attendre dehors. Une page d'air frais reste un peu froide.</t>
+          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est près du jardin, un peu lourd. Le matin, le livre dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a une place, malgré le vent. Il a une place, le matin ! Le quai du tapis peut attendre dehors. Une page d'air frais reste un peu froide.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au matin, la lumière est fraîche, près de la porte. Le sac bleu est près du jardin, un peu lourd. Le matin, le livre dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a une place, malgré le vent. Il a une place, le matin ! Le quai du tapis peut attendre dehors. Une page d'air frais reste un peu froide.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au matin, la lumière est fraîche, près de la porte. Le sac bleu est près du jardin, un peu lourd. Le matin, le livre dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a une place, malgré le vent. Il a une place, le matin ! Le quai du tapis peut attendre dehors. Une page d'air frais reste un peu froide.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est près du jardin, un peu lourd. Le matin, le livre dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a une place, malgré le vent. Il a une place, le matin ! Le quai du tapis peut attendre dehors. Une page d'air frais reste un peu froide. [pause]</t>
+          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est près du jardin, un peu lourd. Le matin, le livre dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a une place, malgré le vent. Il a une place, le matin ! Le quai du tapis peut attendre dehors. Une page d'air frais reste un peu froide. [pause]</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -9652,7 +9652,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino couche le livre, pages vers le fond.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|Le livre a une place, malgré le vent.
 enfant-m|Il a une place, le matin !
 maman|Le quai du tapis peut attendre dehors.
@@ -9870,17 +9870,17 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est près du jardin, un peu lourd. Après la sieste, le livre dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a attendu la dalle, à plat. Il a une place, après la sieste ! Le quai du tapis peut attendre dehors. Le livre de sieste sent la dalle chaude.</t>
+          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est près du jardin, un peu lourd. Après la sieste, le livre dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a attendu la dalle, à plat. Il a une place, après la sieste ! Le quai du tapis peut attendre dehors. Le livre de sieste sent la dalle chaude.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Après la sieste, le rideau fait un carré chaud. Le sac bleu est près du jardin, un peu lourd. Après la sieste, le livre dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a attendu la dalle, à plat. Il a une place, après la sieste ! Le quai du tapis peut attendre dehors. Le livre de sieste sent la dalle chaude.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Après la sieste, le rideau fait un carré chaud. Le sac bleu est près du jardin, un peu lourd. Après la sieste, le livre dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a attendu la dalle, à plat. Il a une place, après la sieste ! Le quai du tapis peut attendre dehors. Le livre de sieste sent la dalle chaude.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est près du jardin, un peu lourd. Après la sieste, le livre dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a attendu la dalle, à plat. Il a une place, après la sieste ! Le quai du tapis peut attendre dehors. Le livre de sieste sent la dalle chaude. [pause]</t>
+          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est près du jardin, un peu lourd. Après la sieste, le livre dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a attendu la dalle, à plat. Il a une place, après la sieste ! Le quai du tapis peut attendre dehors. Le livre de sieste sent la dalle chaude. [pause]</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -10021,7 +10021,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino couche le livre, pages vers le fond.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|Le livre a attendu la dalle, à plat.
 enfant-m|Il a une place, après la sieste !
 maman|Le quai du tapis peut attendre dehors.
@@ -10243,17 +10243,17 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est près du jardin, un peu lourd. Le soir, le livre dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a une place, malgré le portail. Il a une place, le soir ! Le quai du tapis peut attendre dehors. Le livre du soir sent le portail, fermé.</t>
+          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est près du jardin, un peu lourd. Le soir, le livre dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a une place, malgré le portail. Il a une place, le soir ! Le quai du tapis peut attendre dehors. Le livre du soir sent le portail, fermé.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, la lampe allume le tapis, tout près. Le sac bleu est près du jardin, un peu lourd. Le soir, le livre dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a une place, malgré le portail. Il a une place, le soir ! Le quai du tapis peut attendre dehors. Le livre du soir sent le portail, fermé.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, la lampe allume le tapis, tout près. Le sac bleu est près du jardin, un peu lourd. Le soir, le livre dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a une place, malgré le portail. Il a une place, le soir ! Le quai du tapis peut attendre dehors. Le livre du soir sent le portail, fermé.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est près du jardin, un peu lourd. Le soir, le livre dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a une place, malgré le portail. Il a une place, le soir ! Le quai du tapis peut attendre dehors. Le livre du soir sent le portail, fermé. [pause]</t>
+          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est près du jardin, un peu lourd. Le soir, le livre dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a une place, malgré le portail. Il a une place, le soir ! Le quai du tapis peut attendre dehors. Le livre du soir sent le portail, fermé. [pause]</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -10394,7 +10394,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino couche le livre, pages vers le fond.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|Le livre a une place, malgré le portail.
 enfant-m|Il a une place, le soir !
 maman|Le quai du tapis peut attendre dehors.
@@ -11002,17 +11002,17 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est près du jardin, un peu lourd. Le matin, la tasse dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a une place, malgré la goutte. Elle a une place, le matin ! Le quai du tapis peut attendre dehors. La tasse du jardin sonne, au matin clair.</t>
+          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est près du jardin, un peu lourd. Le matin, la tasse dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a une place, malgré la goutte. Elle a une place, le matin ! Le quai du tapis peut attendre dehors. La tasse du jardin sonne, au matin clair.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au matin, la lumière est fraîche, près de la porte. Le sac bleu est près du jardin, un peu lourd. Le matin, la tasse dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a une place, malgré la goutte. Elle a une place, le matin ! Le quai du tapis peut attendre dehors. La tasse du jardin sonne, au matin clair.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au matin, la lumière est fraîche, près de la porte. Le sac bleu est près du jardin, un peu lourd. Le matin, la tasse dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a une place, malgré la goutte. Elle a une place, le matin ! Le quai du tapis peut attendre dehors. La tasse du jardin sonne, au matin clair.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est près du jardin, un peu lourd. Le matin, la tasse dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a une place, malgré la goutte. Elle a une place, le matin ! Le quai du tapis peut attendre dehors. La tasse du jardin sonne, au matin clair. [pause]</t>
+          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est près du jardin, un peu lourd. Le matin, la tasse dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a une place, malgré la goutte. Elle a une place, le matin ! Le quai du tapis peut attendre dehors. La tasse du jardin sonne, au matin clair. [pause]</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -11153,7 +11153,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino niche la tasse, contre le doudou.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|La tasse a une place, malgré la goutte.
 enfant-m|Elle a une place, le matin !
 maman|Le quai du tapis peut attendre dehors.
@@ -11371,17 +11371,17 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est près du jardin, un peu lourd. Après la sieste, la tasse dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a perdu sa goutte, au chaud. Elle a une place, après la sieste ! Le quai du tapis peut attendre dehors. La tasse de sieste a perdu sa goutte.</t>
+          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est près du jardin, un peu lourd. Après la sieste, la tasse dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a perdu sa goutte, au chaud. Elle a une place, après la sieste ! Le quai du tapis peut attendre dehors. La tasse de sieste a perdu sa goutte.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Après la sieste, le rideau fait un carré chaud. Le sac bleu est près du jardin, un peu lourd. Après la sieste, la tasse dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a perdu sa goutte, au chaud. Elle a une place, après la sieste ! Le quai du tapis peut attendre dehors. La tasse de sieste a perdu sa goutte.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Après la sieste, le rideau fait un carré chaud. Le sac bleu est près du jardin, un peu lourd. Après la sieste, la tasse dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a perdu sa goutte, au chaud. Elle a une place, après la sieste ! Le quai du tapis peut attendre dehors. La tasse de sieste a perdu sa goutte.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est près du jardin, un peu lourd. Après la sieste, la tasse dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a perdu sa goutte, au chaud. Elle a une place, après la sieste ! Le quai du tapis peut attendre dehors. La tasse de sieste a perdu sa goutte. [pause]</t>
+          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est près du jardin, un peu lourd. Après la sieste, la tasse dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a perdu sa goutte, au chaud. Elle a une place, après la sieste ! Le quai du tapis peut attendre dehors. La tasse de sieste a perdu sa goutte. [pause]</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -11522,7 +11522,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino niche la tasse, contre le doudou.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|La tasse a perdu sa goutte, au chaud.
 enfant-m|Elle a une place, après la sieste !
 maman|Le quai du tapis peut attendre dehors.
@@ -11744,17 +11744,17 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est près du jardin, un peu lourd. Le soir, la tasse dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a une place, malgré le soir. Elle a une place, le soir ! Le quai du tapis peut attendre dehors. La tasse du soir reflète le portail.</t>
+          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est près du jardin, un peu lourd. Le soir, la tasse dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a une place, malgré le soir. Elle a une place, le soir ! Le quai du tapis peut attendre dehors. La tasse du soir reflète le portail.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, la lampe allume le tapis, tout près. Le sac bleu est près du jardin, un peu lourd. Le soir, la tasse dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a une place, malgré le soir. Elle a une place, le soir ! Le quai du tapis peut attendre dehors. La tasse du soir reflète le portail.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, la lampe allume le tapis, tout près. Le sac bleu est près du jardin, un peu lourd. Le soir, la tasse dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a une place, malgré le soir. Elle a une place, le soir ! Le quai du tapis peut attendre dehors. La tasse du soir reflète le portail.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est près du jardin, un peu lourd. Le soir, la tasse dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a une place, malgré le soir. Elle a une place, le soir ! Le quai du tapis peut attendre dehors. La tasse du soir reflète le portail. [pause]</t>
+          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est près du jardin, un peu lourd. Le soir, la tasse dans le sac ! Le doudou a failli rester dans l'herbe. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a une place, malgré le soir. Elle a une place, le soir ! Le quai du tapis peut attendre dehors. La tasse du soir reflète le portail. [pause]</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -11895,7 +11895,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino niche la tasse, contre le doudou.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|La tasse a une place, malgré le soir.
 enfant-m|Elle a une place, le soir !
 maman|Le quai du tapis peut attendre dehors.
@@ -13261,17 +13261,17 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la chambre, un peu lourd. Le matin, les cubes dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont une place, hors du lit. Ils ont une place, le matin ! Le quai du tapis peut attendre dehors. Un cube de lit brille, sous la dent dorée.</t>
+          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la chambre, un peu lourd. Le matin, les cubes dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont une place, hors du lit. Ils ont une place, le matin ! Le quai du tapis peut attendre dehors. Un cube de lit brille, sous la dent dorée.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la chambre, un peu lourd. Le matin, les cubes dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont une place, hors du lit. Ils ont une place, le matin ! Le quai du tapis peut attendre dehors. Un cube de lit brille, sous la dent dorée.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la chambre, un peu lourd. Le matin, les cubes dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont une place, hors du lit. Ils ont une place, le matin ! Le quai du tapis peut attendre dehors. Un cube de lit brille, sous la dent dorée.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la chambre, un peu lourd. Le matin, les cubes dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont une place, hors du lit. Ils ont une place, le matin ! Le quai du tapis peut attendre dehors. Un cube de lit brille, sous la dent dorée. [pause]</t>
+          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la chambre, un peu lourd. Le matin, les cubes dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont une place, hors du lit. Ils ont une place, le matin ! Le quai du tapis peut attendre dehors. Un cube de lit brille, sous la dent dorée. [pause]</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -13412,7 +13412,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino glisse un cube, puis l'autre, à plat.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|Tes cubes ont une place, hors du lit.
 enfant-m|Ils ont une place, le matin !
 maman|Le quai du tapis peut attendre dehors.
@@ -13630,17 +13630,17 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la chambre, un peu lourd. Après la sieste, les cubes dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont dormi, puis voyagé. Ils ont une place, après la sieste ! Le quai du tapis peut attendre dehors. Un cube de sieste dort, contre le doudou.</t>
+          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la chambre, un peu lourd. Après la sieste, les cubes dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont dormi, puis voyagé. Ils ont une place, après la sieste ! Le quai du tapis peut attendre dehors. Un cube de sieste dort, contre le doudou.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la chambre, un peu lourd. Après la sieste, les cubes dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont dormi, puis voyagé. Ils ont une place, après la sieste ! Le quai du tapis peut attendre dehors. Un cube de sieste dort, contre le doudou.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la chambre, un peu lourd. Après la sieste, les cubes dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont dormi, puis voyagé. Ils ont une place, après la sieste ! Le quai du tapis peut attendre dehors. Un cube de sieste dort, contre le doudou.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la chambre, un peu lourd. Après la sieste, les cubes dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont dormi, puis voyagé. Ils ont une place, après la sieste ! Le quai du tapis peut attendre dehors. Un cube de sieste dort, contre le doudou. [pause]</t>
+          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la chambre, un peu lourd. Après la sieste, les cubes dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont dormi, puis voyagé. Ils ont une place, après la sieste ! Le quai du tapis peut attendre dehors. Un cube de sieste dort, contre le doudou. [pause]</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -13781,7 +13781,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino glisse un cube, puis l'autre, à plat.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|Tes cubes ont dormi, puis voyagé.
 enfant-m|Ils ont une place, après la sieste !
 maman|Le quai du tapis peut attendre dehors.
@@ -14003,17 +14003,17 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la chambre, un peu lourd. Le soir, les cubes dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont une place, sous la lampe. Ils ont une place, le soir ! Le quai du tapis peut attendre dehors. Un cube du soir garde la poussière du lit.</t>
+          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la chambre, un peu lourd. Le soir, les cubes dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont une place, sous la lampe. Ils ont une place, le soir ! Le quai du tapis peut attendre dehors. Un cube du soir garde la poussière du lit.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la chambre, un peu lourd. Le soir, les cubes dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont une place, sous la lampe. Ils ont une place, le soir ! Le quai du tapis peut attendre dehors. Un cube du soir garde la poussière du lit.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la chambre, un peu lourd. Le soir, les cubes dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont une place, sous la lampe. Ils ont une place, le soir ! Le quai du tapis peut attendre dehors. Un cube du soir garde la poussière du lit.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la chambre, un peu lourd. Le soir, les cubes dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent de fermeture dorée glisse, puis tient. Tes cubes ont une place, sous la lampe. Ils ont une place, le soir ! Le quai du tapis peut attendre dehors. Un cube du soir garde la poussière du lit. [pause]</t>
+          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la chambre, un peu lourd. Le soir, les cubes dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino glisse un cube, puis l'autre, à plat. La dent dorée glisse, puis tient. Tes cubes ont une place, sous la lampe. Ils ont une place, le soir ! Le quai du tapis peut attendre dehors. Un cube du soir garde la poussière du lit. [pause]</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr"/>
@@ -14154,7 +14154,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino glisse un cube, puis l'autre, à plat.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|Tes cubes ont une place, sous la lampe.
 enfant-m|Ils ont une place, le soir !
 maman|Le quai du tapis peut attendre dehors.
@@ -14762,17 +14762,17 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la chambre, un peu lourd. Le matin, le livre dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a une place, hors de l'oreiller. Il a une place, le matin ! Le quai du tapis peut attendre dehors. Le livre du matin sent l'oreiller, tiède.</t>
+          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la chambre, un peu lourd. Le matin, le livre dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a une place, hors de l'oreiller. Il a une place, le matin ! Le quai du tapis peut attendre dehors. Le livre du matin sent l'oreiller, tiède.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la chambre, un peu lourd. Le matin, le livre dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a une place, hors de l'oreiller. Il a une place, le matin ! Le quai du tapis peut attendre dehors. Le livre du matin sent l'oreiller, tiède.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la chambre, un peu lourd. Le matin, le livre dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a une place, hors de l'oreiller. Il a une place, le matin ! Le quai du tapis peut attendre dehors. Le livre du matin sent l'oreiller, tiède.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la chambre, un peu lourd. Le matin, le livre dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a une place, hors de l'oreiller. Il a une place, le matin ! Le quai du tapis peut attendre dehors. Le livre du matin sent l'oreiller, tiède. [pause]</t>
+          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la chambre, un peu lourd. Le matin, le livre dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a une place, hors de l'oreiller. Il a une place, le matin ! Le quai du tapis peut attendre dehors. Le livre du matin sent l'oreiller, tiède. [pause]</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
@@ -14913,7 +14913,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino couche le livre, pages vers le fond.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|Le livre a une place, hors de l'oreiller.
 enfant-m|Il a une place, le matin !
 maman|Le quai du tapis peut attendre dehors.
@@ -15131,17 +15131,17 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la chambre, un peu lourd. Après la sieste, le livre dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a attendu le rideau, à plat. Il a une place, après la sieste ! Le quai du tapis peut attendre dehors. Le livre de sieste fait un toit, au lit.</t>
+          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la chambre, un peu lourd. Après la sieste, le livre dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a attendu le rideau, à plat. Il a une place, après la sieste ! Le quai du tapis peut attendre dehors. Le livre de sieste fait un toit, au lit.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la chambre, un peu lourd. Après la sieste, le livre dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a attendu le rideau, à plat. Il a une place, après la sieste ! Le quai du tapis peut attendre dehors. Le livre de sieste fait un toit, au lit.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la chambre, un peu lourd. Après la sieste, le livre dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a attendu le rideau, à plat. Il a une place, après la sieste ! Le quai du tapis peut attendre dehors. Le livre de sieste fait un toit, au lit.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la chambre, un peu lourd. Après la sieste, le livre dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a attendu le rideau, à plat. Il a une place, après la sieste ! Le quai du tapis peut attendre dehors. Le livre de sieste fait un toit, au lit. [pause]</t>
+          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la chambre, un peu lourd. Après la sieste, le livre dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a attendu le rideau, à plat. Il a une place, après la sieste ! Le quai du tapis peut attendre dehors. Le livre de sieste fait un toit, au lit. [pause]</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -15282,7 +15282,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino couche le livre, pages vers le fond.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|Le livre a attendu le rideau, à plat.
 enfant-m|Il a une place, après la sieste !
 maman|Le quai du tapis peut attendre dehors.
@@ -15504,17 +15504,17 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la chambre, un peu lourd. Le soir, le livre dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a une place, hors du pli. Il a une place, le soir ! Le quai du tapis peut attendre dehors. Le livre du soir garde un pli d'oreiller.</t>
+          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la chambre, un peu lourd. Le soir, le livre dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a une place, hors du pli. Il a une place, le soir ! Le quai du tapis peut attendre dehors. Le livre du soir garde un pli d'oreiller.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la chambre, un peu lourd. Le soir, le livre dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a une place, hors du pli. Il a une place, le soir ! Le quai du tapis peut attendre dehors. Le livre du soir garde un pli d'oreiller.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la chambre, un peu lourd. Le soir, le livre dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a une place, hors du pli. Il a une place, le soir ! Le quai du tapis peut attendre dehors. Le livre du soir garde un pli d'oreiller.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la chambre, un peu lourd. Le soir, le livre dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent de fermeture dorée glisse, puis tient. Le livre a une place, hors du pli. Il a une place, le soir ! Le quai du tapis peut attendre dehors. Le livre du soir garde un pli d'oreiller. [pause]</t>
+          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la chambre, un peu lourd. Le soir, le livre dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino couche le livre, pages vers le fond. La dent dorée glisse, puis tient. Le livre a une place, hors du pli. Il a une place, le soir ! Le quai du tapis peut attendre dehors. Le livre du soir garde un pli d'oreiller. [pause]</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
@@ -15655,7 +15655,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino couche le livre, pages vers le fond.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|Le livre a une place, hors du pli.
 enfant-m|Il a une place, le soir !
 maman|Le quai du tapis peut attendre dehors.
@@ -16263,17 +16263,17 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la chambre, un peu lourd. Le matin, la tasse dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a une place, hors du drap. Elle a une place, le matin ! Le quai du tapis peut attendre dehors. La tasse du lit sonne, au matin clair.</t>
+          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la chambre, un peu lourd. Le matin, la tasse dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a une place, hors du drap. Elle a une place, le matin ! Le quai du tapis peut attendre dehors. La tasse du lit sonne, au matin clair.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la chambre, un peu lourd. Le matin, la tasse dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a une place, hors du drap. Elle a une place, le matin ! Le quai du tapis peut attendre dehors. La tasse du lit sonne, au matin clair.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la chambre, un peu lourd. Le matin, la tasse dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a une place, hors du drap. Elle a une place, le matin ! Le quai du tapis peut attendre dehors. La tasse du lit sonne, au matin clair.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la chambre, un peu lourd. Le matin, la tasse dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a une place, hors du drap. Elle a une place, le matin ! Le quai du tapis peut attendre dehors. La tasse du lit sonne, au matin clair. [pause]</t>
+          <t>Au matin, la lumière est fraîche, près de la porte. Le sac bleu est dans la chambre, un peu lourd. Le matin, la tasse dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a une place, hors du drap. Elle a une place, le matin ! Le quai du tapis peut attendre dehors. La tasse du lit sonne, au matin clair. [pause]</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr"/>
@@ -16414,7 +16414,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino niche la tasse, contre le doudou.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|La tasse a une place, hors du drap.
 enfant-m|Elle a une place, le matin !
 maman|Le quai du tapis peut attendre dehors.
@@ -16632,17 +16632,17 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la chambre, un peu lourd. Après la sieste, la tasse dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a attendu, contre le doudou. Elle a une place, après la sieste ! Le quai du tapis peut attendre dehors. La tasse de sieste s'est nichée, au chaud.</t>
+          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la chambre, un peu lourd. Après la sieste, la tasse dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a attendu, contre le doudou. Elle a une place, après la sieste ! Le quai du tapis peut attendre dehors. La tasse de sieste s'est nichée, au chaud.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la chambre, un peu lourd. Après la sieste, la tasse dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a attendu, contre le doudou. Elle a une place, après la sieste ! Le quai du tapis peut attendre dehors. La tasse de sieste s'est nichée, au chaud.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la chambre, un peu lourd. Après la sieste, la tasse dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a attendu, contre le doudou. Elle a une place, après la sieste ! Le quai du tapis peut attendre dehors. La tasse de sieste s'est nichée, au chaud.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la chambre, un peu lourd. Après la sieste, la tasse dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a attendu, contre le doudou. Elle a une place, après la sieste ! Le quai du tapis peut attendre dehors. La tasse de sieste s'est nichée, au chaud. [pause]</t>
+          <t>Après la sieste, le rideau fait un carré chaud. Le sac bleu est dans la chambre, un peu lourd. Après la sieste, la tasse dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a attendu, contre le doudou. Elle a une place, après la sieste ! Le quai du tapis peut attendre dehors. La tasse de sieste s'est nichée, au chaud. [pause]</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
@@ -16783,7 +16783,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino niche la tasse, contre le doudou.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|La tasse a attendu, contre le doudou.
 enfant-m|Elle a une place, après la sieste !
 maman|Le quai du tapis peut attendre dehors.
@@ -17005,17 +17005,17 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la chambre, un peu lourd. Le soir, la tasse dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a une place, sous la lampe. Elle a une place, le soir ! Le quai du tapis peut attendre dehors. La tasse du soir cache un rond de lampe.</t>
+          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la chambre, un peu lourd. Le soir, la tasse dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la dent de fermeture dorée cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a une place, sous la lampe. Elle a une place, le soir ! Le quai du tapis peut attendre dehors. La tasse du soir cache un rond de lampe.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la chambre, un peu lourd. Le soir, la tasse dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a une place, sous la lampe. Elle a une place, le soir ! Le quai du tapis peut attendre dehors. La tasse du soir cache un rond de lampe.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la chambre, un peu lourd. Le soir, la tasse dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis level="moderate"&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a une place, sous la lampe. Elle a une place, le soir ! Le quai du tapis peut attendre dehors. La tasse du soir cache un rond de lampe.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la chambre, un peu lourd. Le soir, la tasse dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent de fermeture dorée glisse, puis tient. La tasse a une place, sous la lampe. Elle a une place, le soir ! Le quai du tapis peut attendre dehors. La tasse du soir cache un rond de lampe. [pause]</t>
+          <t>Le soir, la lampe allume le tapis, tout près. Le sac bleu est dans la chambre, un peu lourd. Le soir, la tasse dans le sac ! La sangle a failli rester sous le lit. Je ne force pas. Il s'arrête, et la &lt;emphasis&gt;dent de fermeture dorée&lt;/emphasis&gt; cligne. Victorino niche la tasse, contre le doudou. La dent dorée glisse, puis tient. La tasse a une place, sous la lampe. Elle a une place, le soir ! Le quai du tapis peut attendre dehors. La tasse du soir cache un rond de lampe. [pause]</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
@@ -17156,7 +17156,7 @@
 enfant-m|Je ne force pas.
 narrateur|Il s'arrête, et la dent de fermeture dorée cligne.
 narrateur|Victorino niche la tasse, contre le doudou.
-narrateur|La dent de fermeture dorée glisse, puis tient.
+narrateur|La dent dorée glisse, puis tient.
 papa|La tasse a une place, sous la lampe.
 enfant-m|Elle a une place, le soir !
 maman|Le quai du tapis peut attendre dehors.
@@ -17368,7 +17368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17425,6 +17425,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>